<commit_message>
feat(template): beautify student class import template with ExcelJS
Rewrote gen-student-class-template.mjs using ExcelJS (matching parent
template style):
- Row 1: dark blue header with bold white text
- Row 2: red hint row marking both fields as required
- Rows 3-4: example data with light background
- Frozen top 2 rows
- Proper column widths
- Added 說明 sheet with 5 usage notes (matching logic, not-found handling,
  ambiguous same-name flow, already-enrolled behavior)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/web/public/assets/templates/student-class-import-template.xlsx
+++ b/apps/web/public/assets/templates/student-class-import-template.xlsx
@@ -1,58 +1,128 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="資料" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="資料" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="說明" state="visible" r:id="rId5"/>
   </sheets>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
+  <si>
+    <t>學生姓名 *</t>
+  </si>
+  <si>
+    <t>就讀學校 *</t>
+  </si>
+  <si>
+    <t>必填</t>
+  </si>
+  <si>
+    <t>陳志遠</t>
+  </si>
+  <si>
+    <t>建國中學</t>
+  </si>
+  <si>
+    <t>林佳慧</t>
+  </si>
+  <si>
+    <t>北一女中</t>
+  </si>
+  <si>
+    <t>注意事項</t>
+  </si>
+  <si>
+    <t>1. 上傳後系統會以「姓名 + 就讀學校」比對現有學生資料</t>
+  </si>
+  <si>
+    <t>2. 若找不到學生，該筆顯示「找不到」，需先至學生管理頁新增</t>
+  </si>
+  <si>
+    <t>3. 同名同校時會顯示下拉選單，請手動選擇正確學生</t>
+  </si>
+  <si>
+    <t>4. 已在班級的學生會顯示「已在班級」並自動略過</t>
+  </si>
+  <si>
+    <t>5. 不需加入的列直接刪除該行即可，無需填任何標記</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <i/>
+      <color rgb="FFCC3300"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <color rgb="FF444444"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF1E3A5F"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <color rgb="FF333333"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1E3A5F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5F5F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFAFAFA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE8EEF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -60,18 +130,85 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF1E3A5F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF1E3A5F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF1E3A5F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF1E3A5F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFDDDDDD"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFDDDDDD"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDDDDDD"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFDDDDDD"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFDDDDDD"/>
+      </right>
+      <top/>
+      <bottom style="hair">
+        <color rgb="FFEEEEEE"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="7">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,36 +533,92 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>學生姓名*</v>
-      </c>
-      <c r="B1" t="str">
-        <v>就讀學校*</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>陳志遠</v>
-      </c>
-      <c r="B2" t="str">
-        <v>建國中學</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>林佳慧</v>
-      </c>
-      <c r="B3" t="str">
-        <v>北一女中</v>
+    <row r="1" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B3"/>
-  </ignoredErrors>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A6"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="52" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>